<commit_message>
Giai đoạn 11.5: detail design Nhân viên, Thêm/Sửa nhân viên, Lịch làm, Cài đặt; hoàn thành GĐ 11
- 14_NhanVien: danh sách tài khoản và tag ca / đã khoá, nhật ký thao tác (lọc thời gian, người,
  xem thêm), quyền cố định của vai trò Nhân viên.
- 15_ThemSuaNhanVien: thông tin cá nhân, tên đăng nhập, mật khẩu tạm (tạo ngẫu nhiên), bắt đổi
  mật khẩu, vai trò, khoá/mở; không tự khoá / tự đổi vai trò; lỗi.
- 16_LichLam: bảng ca theo tuần, ca theo mẫu / ca lẻ / đã sửa giờ, sửa ca, ca mẫu, sao chép tuần
  trước, độ phủ đơn cần nhân viên đón, cảnh báo và ô "Cần người".
- 17_CaiDat: mẫu tin nhắn (mẫu tự chọn sẵn, chèn biến, mã cửa), thông tin homestay.
- Chạy lại toàn bộ công cụ một lần cho 18 file với cùng dữ liệu mẫu; DB dev về đúng baseline.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/detail-design/04_TongQuan.xlsx
+++ b/docs/detail-design/04_TongQuan.xlsx
@@ -707,7 +707,7 @@
       <xdr:row>1</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="9658350" cy="9691885"/>
+    <xdr:ext cx="9658350" cy="9993709"/>
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="1" name="Picture 1">
@@ -743,10 +743,10 @@
     <xdr:from>
       <xdr:col>1</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>55</xdr:row>
+      <xdr:row>57</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="9658350" cy="9564449"/>
+    <xdr:ext cx="9658350" cy="9859565"/>
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="2" name="Picture 2">
@@ -1888,7 +1888,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B1:AG55"/>
+  <dimension ref="B1:AG57"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="2" customWidth="1"/>
@@ -1931,46 +1931,46 @@
       <c r="AF1" s="4"/>
       <c r="AG1" s="4"/>
     </row>
-    <row r="55" ht="21" customHeight="1" spans="2:33" x14ac:dyDescent="0.25">
-      <c r="B55" s="4" t="s">
+    <row r="57" ht="21" customHeight="1" spans="2:33" x14ac:dyDescent="0.25">
+      <c r="B57" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="C55" s="4"/>
-      <c r="D55" s="4"/>
-      <c r="E55" s="4"/>
-      <c r="F55" s="4"/>
-      <c r="G55" s="4"/>
-      <c r="H55" s="4"/>
-      <c r="I55" s="4"/>
-      <c r="J55" s="4"/>
-      <c r="K55" s="4"/>
-      <c r="L55" s="4"/>
-      <c r="M55" s="4"/>
-      <c r="N55" s="4"/>
-      <c r="O55" s="4"/>
-      <c r="P55" s="4"/>
-      <c r="Q55" s="4"/>
-      <c r="R55" s="4"/>
-      <c r="S55" s="4"/>
-      <c r="T55" s="4"/>
-      <c r="U55" s="4"/>
-      <c r="V55" s="4"/>
-      <c r="W55" s="4"/>
-      <c r="X55" s="4"/>
-      <c r="Y55" s="4"/>
-      <c r="Z55" s="4"/>
-      <c r="AA55" s="4"/>
-      <c r="AB55" s="4"/>
-      <c r="AC55" s="4"/>
-      <c r="AD55" s="4"/>
-      <c r="AE55" s="4"/>
-      <c r="AF55" s="4"/>
-      <c r="AG55" s="4"/>
+      <c r="C57" s="4"/>
+      <c r="D57" s="4"/>
+      <c r="E57" s="4"/>
+      <c r="F57" s="4"/>
+      <c r="G57" s="4"/>
+      <c r="H57" s="4"/>
+      <c r="I57" s="4"/>
+      <c r="J57" s="4"/>
+      <c r="K57" s="4"/>
+      <c r="L57" s="4"/>
+      <c r="M57" s="4"/>
+      <c r="N57" s="4"/>
+      <c r="O57" s="4"/>
+      <c r="P57" s="4"/>
+      <c r="Q57" s="4"/>
+      <c r="R57" s="4"/>
+      <c r="S57" s="4"/>
+      <c r="T57" s="4"/>
+      <c r="U57" s="4"/>
+      <c r="V57" s="4"/>
+      <c r="W57" s="4"/>
+      <c r="X57" s="4"/>
+      <c r="Y57" s="4"/>
+      <c r="Z57" s="4"/>
+      <c r="AA57" s="4"/>
+      <c r="AB57" s="4"/>
+      <c r="AC57" s="4"/>
+      <c r="AD57" s="4"/>
+      <c r="AE57" s="4"/>
+      <c r="AF57" s="4"/>
+      <c r="AG57" s="4"/>
     </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="B1:AG1"/>
-    <mergeCell ref="B55:AG55"/>
+    <mergeCell ref="B57:AG57"/>
   </mergeCells>
   <pageSetup paperSize="9" orientation="landscape" fitToWidth="1" fitToHeight="0"/>
   <drawing r:id="rId1"/>

</xml_diff>